<commit_message>
fix: perbaikan import regu
</commit_message>
<xml_diff>
--- a/public/templates/template_regu.xlsx
+++ b/public/templates/template_regu.xlsx
@@ -25,27 +25,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>regu</t>
   </si>
   <si>
+    <t>jenis_kelamin</t>
+  </si>
+  <si>
     <t>Merah</t>
   </si>
   <si>
+    <t>Laki - Laki</t>
+  </si>
+  <si>
     <t>Kuning</t>
   </si>
   <si>
-    <t>Hijau</t>
-  </si>
-  <si>
-    <t>Biru</t>
-  </si>
-  <si>
-    <t>Abu Abu</t>
-  </si>
-  <si>
-    <t>Biru Muda</t>
+    <t>Perempuan</t>
   </si>
 </sst>
 </file>
@@ -362,43 +359,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns:ns0="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" ns0:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ns0:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ns0:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ns0:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ns0:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ns0:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="3" spans="1:2" ns0:dyDescent="0.3">
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>